<commit_message>
Fix AAF differential cap part number (4.7nF -> 47nF)
No.9（C1 = AAF差動C）の型番が GRM3195C1H472JA01D になっていたが、
Murataの容量コード 472 = 47x10^2 pF = 4.7nF であり、必要な 47nF ではない。
このままでは fc が約1.7kHz→約17kHz となり fs/2(3.9kHz) を超えて
アンチエイリアスが破綻するため、473（=47nF）品へ修正。

- E15: GRM3195C1H472JA01D -> C3216C0G1H473J160AA（47nF/C0G/50V/1206）
- F15: Murata -> TDK
- L15: 修正内容と「単価は要再確認」を備考に追記
- F16: C0805C102J5GACTU は KEMET 製のため メーカー表記を修正

「単価入力済み」シートも上記に合わせて再生成。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PCB_STM/README/PMU_部品表_V2_電圧のみ.xlsx
+++ b/PCB_STM/README/PMU_部品表_V2_電圧のみ.xlsx
@@ -385,7 +385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -479,6 +479,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1421,12 +1424,12 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>GRM3195C1H472JA01D</t>
+          <t>C3216C0G1H473J160AA</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>TDK</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1449,7 +1452,7 @@
       </c>
       <c r="L15" s="9" t="inlineStr">
         <is>
-          <t>★473=47nF（472は4.7nFで誤り）／代替 WIMA FKP2</t>
+          <t>★型番修正: GRM3195C1H472JA01D は472=4.7nFで誤り→473=47nFへ変更。単価は要再確認。代替 WIMA FKP2 47nF/63V</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1482,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>KEMET</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -2570,7 +2573,7 @@
       </c>
     </row>
     <row r="5" ht="28" customHeight="1" s="15">
-      <c r="A5" s="41" t="inlineStr">
+      <c r="A5" s="42" t="inlineStr">
         <is>
           <t>Resistor</t>
         </is>
@@ -2580,7 +2583,7 @@
           <t>RG2012P-514-B-T5</t>
         </is>
       </c>
-      <c r="C5" s="41" t="inlineStr">
+      <c r="C5" s="42" t="inlineStr">
         <is>
           <t>Susumu</t>
         </is>
@@ -2602,7 +2605,7 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" s="15">
-      <c r="A6" s="41" t="inlineStr">
+      <c r="A6" s="42" t="inlineStr">
         <is>
           <t>Resistor</t>
         </is>
@@ -2612,7 +2615,7 @@
           <t>RG2012P-512-B-T5</t>
         </is>
       </c>
-      <c r="C6" s="41" t="inlineStr">
+      <c r="C6" s="42" t="inlineStr">
         <is>
           <t>Susumu</t>
         </is>
@@ -2634,7 +2637,7 @@
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" s="15">
-      <c r="A7" s="41" t="inlineStr">
+      <c r="A7" s="42" t="inlineStr">
         <is>
           <t>Resistor</t>
         </is>
@@ -2644,7 +2647,7 @@
           <t>RG2012P-102-B-T5</t>
         </is>
       </c>
-      <c r="C7" s="41" t="inlineStr">
+      <c r="C7" s="42" t="inlineStr">
         <is>
           <t>Susumu</t>
         </is>
@@ -2666,7 +2669,7 @@
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" s="15">
-      <c r="A8" s="41" t="inlineStr">
+      <c r="A8" s="42" t="inlineStr">
         <is>
           <t>MLCC</t>
         </is>
@@ -2676,7 +2679,7 @@
           <t>GCM21BR91H104KA37L</t>
         </is>
       </c>
-      <c r="C8" s="41" t="inlineStr">
+      <c r="C8" s="42" t="inlineStr">
         <is>
           <t>Murata</t>
         </is>
@@ -2698,7 +2701,7 @@
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" s="15">
-      <c r="A9" s="41" t="inlineStr">
+      <c r="A9" s="42" t="inlineStr">
         <is>
           <t>MLCC</t>
         </is>
@@ -2708,7 +2711,7 @@
           <t>GRM219R61H105KA73J</t>
         </is>
       </c>
-      <c r="C9" s="41" t="inlineStr">
+      <c r="C9" s="42" t="inlineStr">
         <is>
           <t>Murata</t>
         </is>
@@ -2730,7 +2733,7 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" s="15">
-      <c r="A10" s="41" t="inlineStr">
+      <c r="A10" s="42" t="inlineStr">
         <is>
           <t>MLCC</t>
         </is>
@@ -2740,7 +2743,7 @@
           <t>GRJ21BR61E106KE01K</t>
         </is>
       </c>
-      <c r="C10" s="41" t="inlineStr">
+      <c r="C10" s="42" t="inlineStr">
         <is>
           <t>Murata</t>
         </is>
@@ -2762,7 +2765,7 @@
       </c>
     </row>
     <row r="11" ht="28" customHeight="1" s="15">
-      <c r="A11" s="41" t="inlineStr">
+      <c r="A11" s="42" t="inlineStr">
         <is>
           <t>Electrolytic Cap</t>
         </is>
@@ -2772,7 +2775,7 @@
           <t>EEU-FR1C101</t>
         </is>
       </c>
-      <c r="C11" s="41" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
         <is>
           <t>Panasonic</t>
         </is>
@@ -2794,7 +2797,7 @@
       </c>
     </row>
     <row r="12" ht="28" customHeight="1" s="15">
-      <c r="A12" s="41" t="inlineStr">
+      <c r="A12" s="42" t="inlineStr">
         <is>
           <t>Electrolytic Cap</t>
         </is>
@@ -2804,7 +2807,7 @@
           <t>UPW1C471MPD6</t>
         </is>
       </c>
-      <c r="C12" s="41" t="inlineStr">
+      <c r="C12" s="42" t="inlineStr">
         <is>
           <t>Nichicon</t>
         </is>
@@ -2826,19 +2829,19 @@
       </c>
     </row>
     <row r="13" ht="28" customHeight="1" s="15">
-      <c r="A13" s="41" t="inlineStr">
+      <c r="A13" s="42" t="inlineStr">
         <is>
           <t>MLCC</t>
         </is>
       </c>
       <c r="B13" s="33" t="inlineStr">
         <is>
-          <t>GRM3195C1H472JA01D</t>
-        </is>
-      </c>
-      <c r="C13" s="41" t="inlineStr">
-        <is>
-          <t>Murata</t>
+          <t>C3216C0G1H473J160AA</t>
+        </is>
+      </c>
+      <c r="C13" s="42" t="inlineStr">
+        <is>
+          <t>TDK</t>
         </is>
       </c>
       <c r="D13" s="34" t="inlineStr">
@@ -2858,7 +2861,7 @@
       </c>
     </row>
     <row r="14" ht="28" customHeight="1" s="15">
-      <c r="A14" s="41" t="inlineStr">
+      <c r="A14" s="42" t="inlineStr">
         <is>
           <t>MLCC</t>
         </is>
@@ -2868,9 +2871,9 @@
           <t>C0805C102J5GACTU</t>
         </is>
       </c>
-      <c r="C14" s="41" t="inlineStr">
-        <is>
-          <t>Murata</t>
+      <c r="C14" s="42" t="inlineStr">
+        <is>
+          <t>KEMET</t>
         </is>
       </c>
       <c r="D14" s="34" t="inlineStr">
@@ -2890,7 +2893,7 @@
       </c>
     </row>
     <row r="15" ht="28" customHeight="1" s="15">
-      <c r="A15" s="41" t="inlineStr">
+      <c r="A15" s="42" t="inlineStr">
         <is>
           <t>IC</t>
         </is>
@@ -2900,7 +2903,7 @@
           <t>AMC3330DWE</t>
         </is>
       </c>
-      <c r="C15" s="41" t="inlineStr">
+      <c r="C15" s="42" t="inlineStr">
         <is>
           <t>Texas Instruments</t>
         </is>
@@ -2922,7 +2925,7 @@
       </c>
     </row>
     <row r="16" ht="28" customHeight="1" s="15">
-      <c r="A16" s="41" t="inlineStr">
+      <c r="A16" s="42" t="inlineStr">
         <is>
           <t>IC</t>
         </is>
@@ -2932,7 +2935,7 @@
           <t>ADS131M02IPWR</t>
         </is>
       </c>
-      <c r="C16" s="41" t="inlineStr">
+      <c r="C16" s="42" t="inlineStr">
         <is>
           <t>Texas Instruments</t>
         </is>
@@ -2954,7 +2957,7 @@
       </c>
     </row>
     <row r="17" ht="28" customHeight="1" s="15">
-      <c r="A17" s="41" t="inlineStr">
+      <c r="A17" s="42" t="inlineStr">
         <is>
           <t>IC</t>
         </is>
@@ -2964,7 +2967,7 @@
           <t>ADP7142AUJZ-3.3-R7</t>
         </is>
       </c>
-      <c r="C17" s="41" t="inlineStr">
+      <c r="C17" s="42" t="inlineStr">
         <is>
           <t>Analog Devices</t>
         </is>
@@ -2986,7 +2989,7 @@
       </c>
     </row>
     <row r="18" ht="28" customHeight="1" s="15">
-      <c r="A18" s="41" t="inlineStr">
+      <c r="A18" s="42" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
@@ -2996,7 +2999,7 @@
           <t>HLK-10M05</t>
         </is>
       </c>
-      <c r="C18" s="41" t="inlineStr">
+      <c r="C18" s="42" t="inlineStr">
         <is>
           <t>Hi-Link</t>
         </is>
@@ -3018,7 +3021,7 @@
       </c>
     </row>
     <row r="19" ht="28" customHeight="1" s="15">
-      <c r="A19" s="41" t="inlineStr">
+      <c r="A19" s="42" t="inlineStr">
         <is>
           <t>Ferrite Bead</t>
         </is>
@@ -3028,7 +3031,7 @@
           <t>BLM31PG601SN1L</t>
         </is>
       </c>
-      <c r="C19" s="41" t="inlineStr">
+      <c r="C19" s="42" t="inlineStr">
         <is>
           <t>Murata</t>
         </is>
@@ -3050,7 +3053,7 @@
       </c>
     </row>
     <row r="20" ht="28" customHeight="1" s="15">
-      <c r="A20" s="41" t="inlineStr">
+      <c r="A20" s="42" t="inlineStr">
         <is>
           <t>Fuse</t>
         </is>
@@ -3060,7 +3063,7 @@
           <t>0215.500MXP</t>
         </is>
       </c>
-      <c r="C20" s="41" t="inlineStr">
+      <c r="C20" s="42" t="inlineStr">
         <is>
           <t>Littelfuse</t>
         </is>
@@ -3082,7 +3085,7 @@
       </c>
     </row>
     <row r="21" ht="28" customHeight="1" s="15">
-      <c r="A21" s="41" t="inlineStr">
+      <c r="A21" s="42" t="inlineStr">
         <is>
           <t>Fuse Holder</t>
         </is>
@@ -3092,7 +3095,7 @@
           <t>0031.8201</t>
         </is>
       </c>
-      <c r="C21" s="41" t="inlineStr">
+      <c r="C21" s="42" t="inlineStr">
         <is>
           <t>Schurter inc.</t>
         </is>
@@ -3110,7 +3113,7 @@
       </c>
     </row>
     <row r="22" ht="28" customHeight="1" s="15">
-      <c r="A22" s="41" t="inlineStr">
+      <c r="A22" s="42" t="inlineStr">
         <is>
           <t>Board</t>
         </is>
@@ -3120,7 +3123,7 @@
           <t>NUCLEO-F446RE</t>
         </is>
       </c>
-      <c r="C22" s="41" t="inlineStr">
+      <c r="C22" s="42" t="inlineStr">
         <is>
           <t>STMicroelectronics</t>
         </is>
@@ -3142,7 +3145,7 @@
       </c>
     </row>
     <row r="23" ht="28" customHeight="1" s="15">
-      <c r="A23" s="41" t="inlineStr">
+      <c r="A23" s="42" t="inlineStr">
         <is>
           <t>Board</t>
         </is>
@@ -3152,7 +3155,7 @@
           <t>ESP32-WROOM-32E 開発ボード</t>
         </is>
       </c>
-      <c r="C23" s="41" t="inlineStr">
+      <c r="C23" s="42" t="inlineStr">
         <is>
           <t>Espressif</t>
         </is>
@@ -3174,7 +3177,7 @@
       </c>
     </row>
     <row r="24" ht="28" customHeight="1" s="15">
-      <c r="A24" s="41" t="inlineStr">
+      <c r="A24" s="42" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
@@ -3184,7 +3187,7 @@
           <t>L76K GPS HAT</t>
         </is>
       </c>
-      <c r="C24" s="41" t="inlineStr">
+      <c r="C24" s="42" t="inlineStr">
         <is>
           <t>Waveshare</t>
         </is>
@@ -3206,7 +3209,7 @@
       </c>
     </row>
     <row r="25" ht="28" customHeight="1" s="15">
-      <c r="A25" s="41" t="inlineStr">
+      <c r="A25" s="42" t="inlineStr">
         <is>
           <t>PCB</t>
         </is>
@@ -3216,7 +3219,7 @@
           <t>（要発注）</t>
         </is>
       </c>
-      <c r="C25" s="41" t="n"/>
+      <c r="C25" s="42" t="n"/>
       <c r="D25" s="34" t="inlineStr">
         <is>
           <t>JLCPCB/Elecrow 等</t>

</xml_diff>